<commit_message>
wip: orifice plate (D20) contract, API, reference cases, corpus tools and web, before integration
A checkpoint of the build workflow's first stages (the contract builder and
the API, independent reference, corpus-tool and web builders), committed so
that a container restart cannot lose them. Integration, review, fixes and
the gates follow in later commits; this commit is not verified.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016WLCGWzpfJ8FCWF7Zv5Uvi
</commit_message>
<xml_diff>
--- a/apps/web/src/lib/utils/__fixtures__/export-results.xlsx
+++ b/apps/web/src/lib/utils/__fixtures__/export-results.xlsx
@@ -365,13 +365,13 @@
     <t>Calculation methods version</t>
   </si>
   <si>
-    <t>1.3.0</t>
+    <t>1.4.0</t>
   </si>
   <si>
     <t>Calculation methods changed</t>
   </si>
   <si>
-    <t>This project was last solved with calculation methods version 1.1.0. These results use version 1.3.0, so some values may differ from the ones it was shared with.</t>
+    <t>This project was last solved with calculation methods version 1.1.0. These results use version 1.4.0, so some values may differ from the ones it was shared with.</t>
   </si>
   <si>
     <t>Server library: CoolProp</t>
@@ -1412,7 +1412,7 @@
     <t>Case: base case</t>
   </si>
   <si>
-    <t>OpenSolve Pipe calculation methods version 1.3.0</t>
+    <t>OpenSolve Pipe calculation methods version 1.4.0</t>
   </si>
   <si>
     <t>Solved: 2026-10-25T12:30:00Z</t>

</xml_diff>